<commit_message>
correct nameRoll to 441
</commit_message>
<xml_diff>
--- a/test-site/nameroll1-value.xlsx
+++ b/test-site/nameroll1-value.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\web-projects\test-site\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C28346FD-F444-4069-A893-DCFBC855D6E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{289CBAE6-A708-4BE0-81D9-7D64A136AA76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{23396267-709B-4E41-9020-7C481B582814}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="443">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="443">
   <si>
     <t>曹正烜</t>
   </si>
@@ -1322,9 +1322,6 @@
     <t>name</t>
   </si>
   <si>
-    <t>roll</t>
-  </si>
-  <si>
     <t>邵麗民</t>
   </si>
   <si>
@@ -1368,6 +1365,9 @@
   </si>
   <si>
     <t>馬孝政</t>
+  </si>
+  <si>
+    <t>rollNumber</t>
   </si>
 </sst>
 </file>
@@ -1816,7 +1816,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B444"/>
+  <dimension ref="A1:B442"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" outlineLevelRow="1"/>
   <cols>
     <col min="2" max="2" width="8.77734375" customWidth="1"/>
@@ -1827,7 +1827,7 @@
         <v>426</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>427</v>
+        <v>442</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="15.6">
@@ -2824,7 +2824,7 @@
     </row>
     <row r="126" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A126" s="5" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="B126" s="3">
         <v>125</v>
@@ -2896,7 +2896,7 @@
     </row>
     <row r="135" spans="1:2" ht="15.6" outlineLevel="1">
       <c r="A135" s="5" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="B135" s="3">
         <v>134</v>
@@ -5232,7 +5232,7 @@
     </row>
     <row r="427" spans="1:2" ht="16.5" customHeight="1">
       <c r="A427" s="4" t="s">
-        <v>400</v>
+        <v>423</v>
       </c>
       <c r="B427" s="3">
         <v>426</v>
@@ -5240,7 +5240,7 @@
     </row>
     <row r="428" spans="1:2" ht="16.5" customHeight="1">
       <c r="A428" s="4" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B428" s="3">
         <v>427</v>
@@ -5248,7 +5248,7 @@
     </row>
     <row r="429" spans="1:2" ht="16.5" customHeight="1">
       <c r="A429" s="4" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="B429" s="3">
         <v>428</v>
@@ -5256,7 +5256,7 @@
     </row>
     <row r="430" spans="1:2" ht="16.5" customHeight="1">
       <c r="A430" s="4" t="s">
-        <v>409</v>
+        <v>429</v>
       </c>
       <c r="B430" s="3">
         <v>429</v>
@@ -5264,7 +5264,7 @@
     </row>
     <row r="431" spans="1:2" ht="16.5" customHeight="1">
       <c r="A431" s="4" t="s">
-        <v>425</v>
+        <v>430</v>
       </c>
       <c r="B431" s="3">
         <v>430</v>
@@ -5272,7 +5272,7 @@
     </row>
     <row r="432" spans="1:2" ht="16.5" customHeight="1">
       <c r="A432" s="4" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="B432" s="3">
         <v>431</v>
@@ -5280,7 +5280,7 @@
     </row>
     <row r="433" spans="1:2" ht="16.5" customHeight="1">
       <c r="A433" s="4" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="B433" s="3">
         <v>432</v>
@@ -5288,7 +5288,7 @@
     </row>
     <row r="434" spans="1:2" ht="16.5" customHeight="1">
       <c r="A434" s="4" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="B434" s="3">
         <v>433</v>
@@ -5296,7 +5296,7 @@
     </row>
     <row r="435" spans="1:2" ht="16.5" customHeight="1">
       <c r="A435" s="4" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B435" s="3">
         <v>434</v>
@@ -5304,7 +5304,7 @@
     </row>
     <row r="436" spans="1:2" ht="16.5" customHeight="1">
       <c r="A436" s="4" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B436" s="3">
         <v>435</v>
@@ -5312,7 +5312,7 @@
     </row>
     <row r="437" spans="1:2" ht="15.75" customHeight="1">
       <c r="A437" s="4" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="B437" s="3">
         <v>436</v>
@@ -5320,7 +5320,7 @@
     </row>
     <row r="438" spans="1:2" ht="15.75" customHeight="1">
       <c r="A438" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="B438" s="3">
         <v>437</v>
@@ -5328,7 +5328,7 @@
     </row>
     <row r="439" spans="1:2" ht="15.75" customHeight="1">
       <c r="A439" s="4" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B439" s="3">
         <v>438</v>
@@ -5336,7 +5336,7 @@
     </row>
     <row r="440" spans="1:2" ht="15.75" customHeight="1">
       <c r="A440" s="4" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B440" s="3">
         <v>439</v>
@@ -5344,7 +5344,7 @@
     </row>
     <row r="441" spans="1:2" ht="15.75" customHeight="1">
       <c r="A441" s="4" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="B441" s="3">
         <v>440</v>
@@ -5352,26 +5352,10 @@
     </row>
     <row r="442" spans="1:2" ht="15.75" customHeight="1">
       <c r="A442" s="4" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="B442" s="3">
         <v>441</v>
-      </c>
-    </row>
-    <row r="443" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A443" s="4" t="s">
-        <v>441</v>
-      </c>
-      <c r="B443" s="3">
-        <v>442</v>
-      </c>
-    </row>
-    <row r="444" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A444" s="4" t="s">
-        <v>442</v>
-      </c>
-      <c r="B444" s="3">
-        <v>443</v>
       </c>
     </row>
   </sheetData>

</xml_diff>